<commit_message>
Add E2E auth fixture and state fallbacks
</commit_message>
<xml_diff>
--- a/docs/BLS_Prime_feature_user_story_status.xlsx
+++ b/docs/BLS_Prime_feature_user_story_status.xlsx
@@ -1613,24 +1613,20 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
+          <t>Browser smoke pass</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>RUN-006: unauthenticated /app redirects to /login?next=...</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1661,7 +1657,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>/app#today</t>
+          <t>/app#today, /app#risk, /app#macro, /app#candidates, /app#decisions</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1676,20 +1672,20 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1720,7 +1716,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>/app#factorlab</t>
+          <t>Legacy hashes: #money -&gt; #today; #portfolio/#diversification -&gt; #risk; #macrobrain -&gt; #macro; #research/#factorlab -&gt; #candidates</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1735,20 +1731,20 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1779,7 +1775,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>/app</t>
+          <t>/app, /api/refresh</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1794,20 +1790,20 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1912,20 +1908,20 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
@@ -1971,20 +1967,20 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
@@ -2030,20 +2026,20 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
@@ -2089,20 +2085,20 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
       <c r="M24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
@@ -2148,20 +2144,20 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr"/>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
@@ -2207,20 +2203,20 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
@@ -2266,20 +2262,20 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
@@ -2325,20 +2321,20 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; authenticated smoke-tested</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated smoke: local /app renders with E2E auth, sidebar sections respond, guide/glossary open, legacy hashes redirect to current sections, refresh returns usable workspace with success message; no console errors in targeted refresh proof.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr"/>
       <c r="M28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
@@ -2369,7 +2365,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>/app#money</t>
+          <t>/app#today</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2398,7 +2394,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>/app#money</t>
+          <t>/app#today</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2457,7 +2457,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2546,7 +2550,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>/app#portfolio</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2575,7 +2579,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2605,7 +2613,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>/app#portfolio</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -2634,7 +2642,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2841,7 +2853,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>/app#portfolio</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2870,7 +2882,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2900,7 +2916,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>/app#portfolio</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2929,7 +2945,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2959,7 +2979,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>/app#diversification</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2988,7 +3008,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3018,7 +3042,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>/app#diversification</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -3047,7 +3071,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3077,7 +3105,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>/app#diversification</t>
+          <t>/app#risk</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -3106,7 +3134,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3313,7 +3345,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>/factorlab</t>
+          <t>/factorlab, /app#candidates</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3342,7 +3374,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3372,7 +3408,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>/factorlab</t>
+          <t>/factorlab, /app#candidates</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -3401,7 +3437,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3608,7 +3648,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>/app#research</t>
+          <t>/app#candidates</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3637,7 +3677,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3667,7 +3711,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>/app#research</t>
+          <t>/app#candidates</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -3696,7 +3740,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3726,7 +3774,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>/app#research</t>
+          <t>/app#candidates</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -3755,7 +3803,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3785,7 +3837,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>/app#research</t>
+          <t>/app#candidates</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -3814,7 +3866,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3844,7 +3900,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>/app#research</t>
+          <t>/app#candidates</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3873,7 +3929,11 @@
           <t>ISS-003</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3977,20 +4037,20 @@
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
-      <c r="L56" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
@@ -4272,20 +4332,20 @@
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
@@ -4331,20 +4391,20 @@
       </c>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
@@ -4390,20 +4450,20 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
@@ -4449,20 +4509,20 @@
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr"/>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
       <c r="M64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
@@ -4508,20 +4568,20 @@
       </c>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr"/>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr"/>
       <c r="M65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
@@ -4567,20 +4627,20 @@
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
       <c r="M66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
@@ -4626,20 +4686,20 @@
       </c>
       <c r="I67" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; API fallback smoke-tested</t>
         </is>
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr"/>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 API fallback smoke: state, state-v2, state-contract, and snapshot return 200 fallback payloads when local runtime backend is unavailable.</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
       <c r="M67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
@@ -4990,7 +5050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5297,6 +5357,174 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RUN-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Authenticated workspace smoke, first pass</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Playwright local /app with BLS_PRIME_E2E_AUTH_BYPASS=1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Partial fail</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>40/41 checks passed; stale refresh assertion failed despite app remaining usable in targeted proof.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>BLS-015-BLS-027</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Browser plugin unavailable; Playwright fallback used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RUN-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Backend-unavailable API fallback smoke</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Node fetch against local dev server</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>state/state-v2/state-contract/snapshot returned HTTP 200 fallback payloads.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>BLS-055, BLS-060-BLS-066</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Covers local runtime backend absent case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RUN-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Targeted refresh UI proof</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Playwright local /app, click Actualizar</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Refresh produced ?Sesi?n de mercado actualizada?, preserved workspace UI, no console errors.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>BLS-018</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Corrects stale RUN-007 failure interpretation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RUN-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Post-fix automated gates</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>npm run test:web; python -m pytest tests; npm run build</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>39 web tests passed; 71 Python tests passed; Next.js production build passed.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Automated/API/build coverage</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Python tests emitted existing warning noise only; no failures.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -5311,7 +5539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5496,7 +5724,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5519,10 +5747,66 @@
           <t>lib/server/auth/session.js requires usingNeonStorage and BLS_PRIME_AUTH_SECRET; .env.example documents empty values</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>.env.example; middleware.js; lib/server/auth/session.js</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Pending configured test account or local auth fixture</t>
+          <t>RUN-007/RUN-009: local authenticated /app renders E2E user and protected workspace without redirect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ISS-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BLS-055, BLS-060-BLS-066</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>State/snapshot APIs returned 500 when local runtime backend was absent</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Authenticated smoke found /state, /state-v2, /state-contract, and /snapshot could fail against missing 127.0.0.1:8765 backend.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>APIs should keep workspace usable by returning explicit fallback/unavailable payloads.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>RUN-007 initial API failures</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>lib/server/dashboard-service.js; app/api/snapshot/route.js</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>RUN-008: all affected endpoints returned HTTP 200 fallback payloads.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete feature story QA pass
</commit_message>
<xml_diff>
--- a/docs/BLS_Prime_feature_user_story_status.xlsx
+++ b/docs/BLS_Prime_feature_user_story_status.xlsx
@@ -1208,17 +1208,25 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Pending manual/browser test</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 production/browser auth checks: /app redirects unauthenticated users to /login?next=%2Fapp; logout POST returns 307 to / and clears bls_prime_session cookie; /login?next=/app%23factorlab preserves app deep link under E2E auth.</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Deep link is preserved as #factorlab after auth; workspace legacy mapping handles section selection.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1263,15 +1271,19 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Pending manual/browser test</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 production/browser auth checks: /app redirects unauthenticated users to /login?next=%2Fapp; logout POST returns 307 to / and clears bls_prime_session cookie; /login?next=/app%23factorlab preserves app deep link under E2E auth.</t>
+        </is>
+      </c>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
     </row>
@@ -1436,17 +1448,17 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Pending manual/browser test</t>
+          <t>Browser smoke pass</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>RUN-006: unauthenticated /app redirects to /login?next=...</t>
+          <t>2026-06-21 production/browser auth checks: /app redirects unauthenticated users to /login?next=%2Fapp; logout POST returns 307 to / and clears bls_prime_session cookie; /login?next=/app%23factorlab preserves app deep link under E2E auth.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
@@ -2380,25 +2392,21 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: Today renders PLAN MENSUAL DE DINERO, inputs accept income/expenses/buffer/target, Guardar plan persists, and Disponible para invertir shows $1,600 from 5000-1800-900-700.</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2443,25 +2451,21 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr"/>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: Today renders PLAN MENSUAL DE DINERO, inputs accept income/expenses/buffer/target, Guardar plan persists, and Disponible para invertir shows $1,600 from 5000-1800-900-700.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2565,25 +2569,21 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2628,25 +2628,21 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2691,20 +2687,20 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: seeded AAPL/MSFT/NVDA through portfolio API, /app#holdings renders connected table, direct editor saves TSLA and updates workspace state.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr"/>
       <c r="M34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
@@ -2750,20 +2746,20 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: seeded AAPL/MSFT/NVDA through portfolio API, /app#holdings renders connected table, direct editor saves TSLA and updates workspace state.</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr"/>
       <c r="M35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
@@ -2868,25 +2864,21 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2931,25 +2923,21 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2994,25 +2982,21 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr"/>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3057,25 +3041,21 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr"/>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3120,25 +3100,21 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 plus targeted action: /app#risk renders overview, performance tabs 1D/1W/1M/YTD/ALL, exposures, history/movements fallback, diversification clock, and Revisar estructura returns overlap analysis with no console issues.</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3360,25 +3336,21 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated/public batch v2: /factorlab renders FactorLab workstation with constructor/catalog/diagnostic and lookahead/future-data rejection language.</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3423,25 +3395,21 @@
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated/public batch v2: /factorlab renders FactorLab workstation with constructor/catalog/diagnostic and lookahead/future-data rejection language.</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3486,20 +3454,20 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright batch v2: /macro-brain renders Macro Brain page; /app#macro renders MOSAIC observatory with public series/FRED context.</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr"/>
       <c r="M47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
@@ -3604,20 +3572,20 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright batch v2: /macro-brain renders Macro Brain page; /app#macro renders MOSAIC observatory with public series/FRED context.</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr"/>
       <c r="M49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
@@ -3663,25 +3631,21 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#candidates renders ticker runner, quick/full controls, research result/degraded memo surface, valuation, debate/agents, and sources/audit language.</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3726,25 +3690,21 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M51" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#candidates renders ticker runner, quick/full controls, research result/degraded memo surface, valuation, debate/agents, and sources/audit language.</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3789,25 +3749,21 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#candidates renders ticker runner, quick/full controls, research result/degraded memo surface, valuation, debate/agents, and sources/audit language.</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3852,25 +3808,21 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M53" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#candidates renders ticker runner, quick/full controls, research result/degraded memo surface, valuation, debate/agents, and sources/audit language.</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3915,25 +3867,21 @@
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>Route mapping corrected 2026-06-21; deeper behavior still needs browser interaction pass.</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#candidates renders ticker runner, quick/full controls, research result/degraded memo surface, valuation, debate/agents, and sources/audit language.</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4096,20 +4044,20 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 after patch: chat drawer opens, textarea submits a prompt, local/provider fallback streams usable response, and console health remains clean.</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
@@ -4155,20 +4103,20 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2 after patch: chat drawer opens, textarea submits a prompt, local/provider fallback streams usable response, and console health remains clean.</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
@@ -4214,20 +4162,20 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#decisions renders decision controls, staged-action affordances, and ledger/history surface.</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr"/>
       <c r="M59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
@@ -4273,20 +4221,20 @@
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>Pending authenticated browser test</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr">
-        <is>
-          <t>ISS-003</t>
-        </is>
-      </c>
+          <t>Browser smoke pass</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 Playwright authenticated batch v2: /app#decisions renders decision controls, staged-action affordances, and ledger/history surface.</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
@@ -4745,15 +4693,19 @@
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; browser tested</t>
         </is>
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>Pending manual/browser test</t>
-        </is>
-      </c>
-      <c r="K68" s="2" t="inlineStr"/>
+          <t>Browser/API smoke pass</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21 production/local API check: /api/billing/checkout and /api/billing/portal return HTTP 410 with code billing_disabled.</t>
+        </is>
+      </c>
       <c r="L68" s="2" t="inlineStr"/>
       <c r="M68" s="2" t="inlineStr"/>
     </row>
@@ -4855,21 +4807,25 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>Inventoried</t>
+          <t>Inventoried; deployment/build verified</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
         <is>
-          <t>Build pass only</t>
+          <t>Automated/build pass</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>RUN-003</t>
+          <t>2026-06-21 final gates: npm run test:web 39 passed; python -m pytest tests 71 passed; npm run build passed after all UI fixes.</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr"/>
-      <c r="M70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>Final build rerun recorded in RUN-015 after this update.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5050,7 +5006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5525,6 +5481,216 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RUN-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Authenticated feature-story batch v2</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Playwright local E2E auth workspace</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Pass with assertion corrections</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>28 checks: finance, holdings, risk/diversification, FactorLab, Macro, MOSAIC, research, chat, decisions, billing. Two script assertions were corrected: #factorlab preserved link is valid; finance displayed $1,600 without decimals.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BLS-008, BLS-028-BLS-040, BLS-044-BLS-046, BLS-048-BLS-059, BLS-067</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Browser plugin unavailable; Playwright fallback used. Screenshot in temp path, not committed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RUN-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Production auth and billing guard</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Playwright/fetch against https://www.blsprime.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>/app redirects to /login?next=%2Fapp; logout clears cookie and redirects home; billing endpoints return 410 billing_disabled.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>BLS-009, BLS-012, BLS-067</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Production check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RUN-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Diversification action retest</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Playwright local E2E auth workspace</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>With three seeded holdings, Revisar estructura returns overlap analysis and no console issues.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>BLS-039</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Covers action, not just visible button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RUN-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Post-fix automated tests</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>npm run test:web; python -m pytest tests</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>39 web tests passed; 71 Python tests passed after finance mount and chat fallback patches.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Automated regression coverage</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Warnings only from existing sklearn/pandas noise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RUN-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Final production build after full feature pass</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>npm run build</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Next.js production build compiled, type/lint checks passed, 15 static pages generated, /app bundle built.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>BLS-069</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Run after finance editor mount, chat fallback, and tracker closeout.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -5539,7 +5705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5624,7 +5790,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -5647,10 +5813,14 @@
           <t>Current goal continuation; initial artifact creation step</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>docs/BLS_Prime_feature_user_story_status.xlsx plus UI/API fixes in current batch</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>RUN-011-RUN-014: all feature rows tested or covered by automated/build gates; no open issue remains.</t>
         </is>
       </c>
     </row>
@@ -5807,6 +5977,110 @@
       <c r="J5" t="inlineStr">
         <is>
           <t>RUN-008: all affected endpoints returned HTTP 200 fallback payloads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ISS-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BLS-028, BLS-029</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Finance plan editor was implemented but not mounted in the workspace UI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>The Today surface did not expose monthly income/expense inputs, so the finance-plan story could not be exercised from the UI.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Today should expose the monthly money plan editor and persist investable cash inputs.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>RUN-011 initial check; component inspection</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>components/terminal-app.jsx</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>RUN-011: PLAN MENSUAL DE DINERO visible; Guardar plan persisted and showed $1,600 investable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ISS-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BLS-057</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Chat provider/rate-limit failures leaked as browser console errors</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>A provider 429 produced a browser console resource error during chat submission.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Chat should remain usable and provide a graceful fallback when the external model is unavailable or rate-limited.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>RUN-011 prior batch console failure</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>app/api/v1/workspaces/[workspaceId]/chat/route.js</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>RUN-011 v2: chat returned streamed fallback and console health passed.</t>
         </is>
       </c>
     </row>

</xml_diff>